<commit_message>
Modulo permisos de usuarios
</commit_message>
<xml_diff>
--- a/data/valores_diarios.xlsx
+++ b/data/valores_diarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WinterOS\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE399654-AD06-4772-9B9C-EAF4E996A16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9ABFA8F-0649-4005-A556-B8B8067230A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="5">
   <si>
     <t>DISCO</t>
   </si>
@@ -45,8 +45,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="166" formatCode="\$\ #,##0.00"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="165" formatCode="\$\ #,##0.00"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -114,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -122,16 +122,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -436,7 +442,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -668,6 +674,118 @@
         <v>4</v>
       </c>
     </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="5">
+        <v>93</v>
+      </c>
+      <c r="B17" s="3">
+        <v>46274</v>
+      </c>
+      <c r="C17" s="6">
+        <v>2</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="5">
+        <v>93</v>
+      </c>
+      <c r="B18" s="3">
+        <v>46275</v>
+      </c>
+      <c r="C18" s="6">
+        <v>1</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="5">
+        <v>93</v>
+      </c>
+      <c r="B19" s="3">
+        <v>46276</v>
+      </c>
+      <c r="C19" s="6">
+        <v>4</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="7">
+        <v>65</v>
+      </c>
+      <c r="B20" s="3">
+        <v>46277</v>
+      </c>
+      <c r="C20" s="8">
+        <v>2</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="7">
+        <v>65</v>
+      </c>
+      <c r="B21" s="3">
+        <v>46278</v>
+      </c>
+      <c r="C21" s="8">
+        <v>1</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="7">
+        <v>65</v>
+      </c>
+      <c r="B22" s="3">
+        <v>46279</v>
+      </c>
+      <c r="C22" s="8">
+        <v>3</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="7">
+        <v>24</v>
+      </c>
+      <c r="B23" s="3">
+        <v>46280</v>
+      </c>
+      <c r="C23" s="8">
+        <v>1</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="7">
+        <v>24</v>
+      </c>
+      <c r="B24" s="3">
+        <v>46281</v>
+      </c>
+      <c r="C24" s="8">
+        <v>2</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D4" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Actualiza pagos y funciones del sistema
</commit_message>
<xml_diff>
--- a/data/valores_diarios.xlsx
+++ b/data/valores_diarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WinterOS\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95E2BDF6-0B8B-4115-8508-09CBFC0DDFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAE33690-6B4C-48D3-AB1D-EF9F1A8D5DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="5">
   <si>
     <t>DISCO</t>
   </si>
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -784,7 +784,32 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" s="7"/>
+      <c r="A25" s="5">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3">
+        <v>46282</v>
+      </c>
+      <c r="C25" s="6">
+        <v>2</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" s="7">
+        <v>24</v>
+      </c>
+      <c r="B26" s="3">
+        <v>46283</v>
+      </c>
+      <c r="C26" s="6">
+        <v>2</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D4" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
Modificacion de interfaz de la app
</commit_message>
<xml_diff>
--- a/data/valores_diarios.xlsx
+++ b/data/valores_diarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WinterOS\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAE33690-6B4C-48D3-AB1D-EF9F1A8D5DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95E2BDF6-0B8B-4115-8508-09CBFC0DDFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="5">
   <si>
     <t>DISCO</t>
   </si>
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -784,32 +784,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" s="5">
-        <v>24</v>
-      </c>
-      <c r="B25" s="3">
-        <v>46282</v>
-      </c>
-      <c r="C25" s="6">
-        <v>2</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" s="7">
-        <v>24</v>
-      </c>
-      <c r="B26" s="3">
-        <v>46283</v>
-      </c>
-      <c r="C26" s="6">
-        <v>2</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>4</v>
-      </c>
+      <c r="A25" s="7"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D4" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>